<commit_message>
P4: add weight build-up tab and link take-off mass
</commit_message>
<xml_diff>
--- a/RC-Plane/P4_bom/P4_RC_plane_BOM.xlsx
+++ b/RC-Plane/P4_bom/P4_RC_plane_BOM.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Component Options" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Configurations" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Engineering Checks" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Weight Build-up" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="318">
   <si>
     <t xml:space="preserve">P4 — RC Aircraft Bill of Materials: Component Options</t>
   </si>
@@ -600,7 +601,7 @@
     <t xml:space="preserve">All-up mass</t>
   </si>
   <si>
-    <t xml:space="preserve">Weight build-up spreadsheet (P3)</t>
+    <t xml:space="preserve">Linked from the Weight Build-up tab</t>
   </si>
   <si>
     <t xml:space="preserve">Wing area</t>
@@ -799,19 +800,199 @@
   </si>
   <si>
     <t xml:space="preserve">n × I_servo + I_rx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC Aircraft Weight Build-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bottom-up estimate of the all-up weight. Blue = input, black = formula, green = linked input.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payload (g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumed mission payload (not from the Techfest rulebook)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design all-up weight (g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculated all-up weight rounded up for build margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spar outer diameter (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 × 4 mm pultruded carbon tube (Robu listing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spar inner diameter (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robu listing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spar length (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two 500 mm tubes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carbon fibre density (g/cm³)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical for pultruded carbon fibre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foam board sheet weight (g per 20×30 in sheet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimate for paper-faced foam board; weigh one sheet to confirm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foam sheets used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wing ≈ 1.5 sheets + fuselage and tail ≈ 1 sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spar cross-section area (mm²)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spar mass (g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">area × length ÷ 1000 × density</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit weight (g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total weight (g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% of empty weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source / notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3S 2200 mAh 40C LiPo battery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electronics &amp; battery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robu listing, 175 g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG90 9 g servo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probots listing, 9 g each</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A2212 1000 KV motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thingbits listing ≈ 52 g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 A ESC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical spec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FS-iA6B receiver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carbon fibre spar 6×4 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From spar inputs above</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foam board (paper-faced, 5 mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avoid PVC sunboard — much heavier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hot glue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardware &amp; assembly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Landing gear (steel wire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wires and XT60 connectors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control horns and pushrods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empty weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All-up weight (calculated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design weight used for sizing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margin for build errors (g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margin (% of design weight)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary by category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weight (g)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\₹#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="0.00"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -919,6 +1100,22 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -995,16 +1192,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="56">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1044,15 +1245,95 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1060,23 +1341,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1084,39 +1349,71 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1375,834 +1672,834 @@
   <dimension ref="A1:I31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="6" t="n">
         <v>4999</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="6" t="n">
         <v>2413</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+    <row r="7" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="6" t="n">
         <v>383</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="6" t="n">
         <v>1345</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="6" t="n">
         <v>499</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="6" t="n">
         <v>1038</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+    <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="6" t="n">
         <v>105</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+    <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="6" t="n">
         <v>265</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="6" t="n">
         <v>1444</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="6" t="n">
         <v>1599</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="H14" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+    <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="6" t="n">
         <v>119</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="6" t="s">
+      <c r="H15" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+    <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="6" t="n">
         <v>179</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="H16" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="6" t="n">
         <v>3499</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="H17" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="6" t="n">
         <v>499</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H18" s="6" t="s">
+      <c r="H18" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="6" t="n">
         <v>146</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="H19" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+    <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="6" t="n">
         <v>249</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="H20" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I20" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+    <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="6" t="n">
         <v>299</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="I21" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+    <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="H22" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+    <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="6" t="n">
         <v>95</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="H23" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+    <row r="24" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="H24" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+    <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="6" t="n">
         <v>659</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H25" s="6" t="s">
+      <c r="H25" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I25" s="4" t="s">
+      <c r="I25" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+    <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="H26" s="6" t="s">
+      <c r="H26" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I26" s="7" t="s">
+      <c r="I26" s="8" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="6" t="s">
+      <c r="H27" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I27" s="7" t="s">
+      <c r="I27" s="8" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="H28" s="6" t="s">
+      <c r="H28" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I28" s="7" t="s">
+      <c r="I28" s="8" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="6" t="n">
         <v>350</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="G29" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="H29" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I29" s="7" t="s">
+      <c r="I29" s="8" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="H30" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I30" s="7" t="s">
+      <c r="I30" s="8" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="E31" s="4"/>
-      <c r="F31" s="5" t="n">
+      <c r="E31" s="5"/>
+      <c r="F31" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="H31" s="6" t="s">
+      <c r="H31" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I31" s="7" t="s">
+      <c r="I31" s="8" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2225,815 +2522,815 @@
   <dimension ref="A1:I39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="9" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="11" t="n">
         <f aca="false">'Component Options'!$F$6</f>
         <v>2413</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="12" t="n">
         <f aca="false">C5*D5</f>
         <v>2413</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="11" t="n">
         <f aca="false">'Component Options'!$F$5</f>
         <v>4999</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I5" s="12" t="n">
         <f aca="false">G5*H5</f>
         <v>4999</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="11" t="n">
         <f aca="false">'Component Options'!$F$7</f>
         <v>383</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="12" t="n">
         <f aca="false">C6*D6</f>
         <v>383</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="11" t="n">
         <f aca="false">'Component Options'!$F$8</f>
         <v>1345</v>
       </c>
-      <c r="I6" s="11" t="n">
+      <c r="I6" s="12" t="n">
         <f aca="false">G6*H6</f>
         <v>1345</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <f aca="false">'Component Options'!$F$9</f>
         <v>499</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="12" t="n">
         <f aca="false">C7*D7</f>
         <v>499</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="11" t="n">
         <f aca="false">'Component Options'!$F$10</f>
         <v>1038</v>
       </c>
-      <c r="I7" s="11" t="n">
+      <c r="I7" s="12" t="n">
         <f aca="false">G7*H7</f>
         <v>1038</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="11" t="n">
         <f aca="false">'Component Options'!$F$11</f>
         <v>105</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="12" t="n">
         <f aca="false">C8*D8</f>
         <v>105</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="11" t="n">
         <f aca="false">'Component Options'!$F$12</f>
         <v>265</v>
       </c>
-      <c r="I8" s="11" t="n">
+      <c r="I8" s="12" t="n">
         <f aca="false">G8*H8</f>
         <v>265</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <f aca="false">'Component Options'!$F$13</f>
         <v>1444</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="12" t="n">
         <f aca="false">C9*D9</f>
         <v>1444</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="11" t="n">
         <f aca="false">'Component Options'!$F$13</f>
         <v>1444</v>
       </c>
-      <c r="I9" s="11" t="n">
+      <c r="I9" s="12" t="n">
         <f aca="false">G9*H9</f>
         <v>2888</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="11" t="n">
         <f aca="false">'Component Options'!$F$15</f>
         <v>119</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="12" t="n">
         <f aca="false">C10*D10</f>
         <v>476</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="11" t="n">
         <f aca="false">'Component Options'!$F$16</f>
         <v>179</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="12" t="n">
         <f aca="false">G10*H10</f>
         <v>716</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="11" t="n">
         <f aca="false">'Component Options'!$F$18</f>
         <v>499</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="12" t="n">
         <f aca="false">C11*D11</f>
         <v>499</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="11" t="n">
         <f aca="false">'Component Options'!$F$17</f>
         <v>3499</v>
       </c>
-      <c r="I11" s="11" t="n">
+      <c r="I11" s="12" t="n">
         <f aca="false">G11*H11</f>
         <v>3499</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+    <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="11" t="n">
         <f aca="false">'Component Options'!$F$19</f>
         <v>146</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="12" t="n">
         <f aca="false">C12*D12</f>
         <v>292</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G12" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="H12" s="11" t="n">
         <f aca="false">'Component Options'!$F$20</f>
         <v>249</v>
       </c>
-      <c r="I12" s="11" t="n">
+      <c r="I12" s="12" t="n">
         <f aca="false">G12*H12</f>
         <v>996</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+    <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="11" t="n">
         <f aca="false">'Component Options'!$F$21</f>
         <v>299</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="12" t="n">
         <f aca="false">C13*D13</f>
         <v>299</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="10" t="n">
+      <c r="H13" s="11" t="n">
         <f aca="false">'Component Options'!$F$21</f>
         <v>299</v>
       </c>
-      <c r="I13" s="11" t="n">
+      <c r="I13" s="12" t="n">
         <f aca="false">G13*H13</f>
         <v>299</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+    <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="11" t="n">
         <f aca="false">'Component Options'!$F$22</f>
         <v>49</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="12" t="n">
         <f aca="false">C14*D14</f>
         <v>98</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="10" t="n">
+      <c r="H14" s="11" t="n">
         <f aca="false">'Component Options'!$F$22</f>
         <v>49</v>
       </c>
-      <c r="I14" s="11" t="n">
+      <c r="I14" s="12" t="n">
         <f aca="false">G14*H14</f>
         <v>98</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C15" s="9" t="n">
+      <c r="C15" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="11" t="n">
         <f aca="false">'Component Options'!$F$23</f>
         <v>95</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="12" t="n">
         <f aca="false">C15*D15</f>
         <v>190</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G15" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H15" s="10" t="n">
+      <c r="H15" s="11" t="n">
         <f aca="false">'Component Options'!$F$23</f>
         <v>95</v>
       </c>
-      <c r="I15" s="11" t="n">
+      <c r="I15" s="12" t="n">
         <f aca="false">G15*H15</f>
         <v>190</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D16" s="11" t="n">
         <f aca="false">'Component Options'!$F$24</f>
         <v>39</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="12" t="n">
         <f aca="false">C16*D16</f>
         <v>78</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G16" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="10" t="n">
+      <c r="H16" s="11" t="n">
         <f aca="false">'Component Options'!$F$24</f>
         <v>39</v>
       </c>
-      <c r="I16" s="11" t="n">
+      <c r="I16" s="12" t="n">
         <f aca="false">G16*H16</f>
         <v>78</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="11" t="n">
         <f aca="false">'Component Options'!$F$25</f>
         <v>659</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="12" t="n">
         <f aca="false">C17*D17</f>
         <v>659</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="10" t="n">
+      <c r="H17" s="11" t="n">
         <f aca="false">'Component Options'!$F$25</f>
         <v>659</v>
       </c>
-      <c r="I17" s="11" t="n">
+      <c r="I17" s="12" t="n">
         <f aca="false">G17*H17</f>
         <v>659</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D18" s="11" t="n">
         <f aca="false">'Component Options'!$F$26</f>
         <v>120</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="12" t="n">
         <f aca="false">C18*D18</f>
         <v>480</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="G18" s="9" t="n">
+      <c r="G18" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="H18" s="10" t="n">
+      <c r="H18" s="11" t="n">
         <f aca="false">'Component Options'!$F$26</f>
         <v>120</v>
       </c>
-      <c r="I18" s="11" t="n">
+      <c r="I18" s="12" t="n">
         <f aca="false">G18*H18</f>
         <v>480</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="11" t="n">
         <f aca="false">'Component Options'!$F$27</f>
         <v>300</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="12" t="n">
         <f aca="false">C19*D19</f>
         <v>300</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="G19" s="9" t="n">
+      <c r="G19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="10" t="n">
+      <c r="H19" s="11" t="n">
         <f aca="false">'Component Options'!$F$27</f>
         <v>300</v>
       </c>
-      <c r="I19" s="11" t="n">
+      <c r="I19" s="12" t="n">
         <f aca="false">G19*H19</f>
         <v>300</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="11" t="n">
         <f aca="false">'Component Options'!$F$28</f>
         <v>100</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="12" t="n">
         <f aca="false">C20*D20</f>
         <v>100</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G20" s="9" t="n">
+      <c r="G20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="10" t="n">
+      <c r="H20" s="11" t="n">
         <f aca="false">'Component Options'!$F$28</f>
         <v>100</v>
       </c>
-      <c r="I20" s="11" t="n">
+      <c r="I20" s="12" t="n">
         <f aca="false">G20*H20</f>
         <v>100</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="11" t="n">
         <f aca="false">'Component Options'!$F$29</f>
         <v>350</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="12" t="n">
         <f aca="false">C21*D21</f>
         <v>350</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="G21" s="9" t="n">
+      <c r="G21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="10" t="n">
+      <c r="H21" s="11" t="n">
         <f aca="false">'Component Options'!$F$29</f>
         <v>350</v>
       </c>
-      <c r="I21" s="11" t="n">
+      <c r="I21" s="12" t="n">
         <f aca="false">G21*H21</f>
         <v>350</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="10" t="n">
+      <c r="D22" s="11" t="n">
         <f aca="false">'Component Options'!$F$30</f>
         <v>100</v>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="12" t="n">
         <f aca="false">C22*D22</f>
         <v>100</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="9" t="n">
+      <c r="G22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="10" t="n">
+      <c r="H22" s="11" t="n">
         <f aca="false">'Component Options'!$F$30</f>
         <v>100</v>
       </c>
-      <c r="I22" s="11" t="n">
+      <c r="I22" s="12" t="n">
         <f aca="false">G22*H22</f>
         <v>100</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="10" t="n">
+      <c r="D23" s="11" t="n">
         <f aca="false">'Component Options'!$F$31</f>
         <v>150</v>
       </c>
-      <c r="E23" s="11" t="n">
+      <c r="E23" s="12" t="n">
         <f aca="false">C23*D23</f>
         <v>150</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="G23" s="9" t="n">
+      <c r="G23" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="10" t="n">
+      <c r="H23" s="11" t="n">
         <f aca="false">'Component Options'!$F$31</f>
         <v>150</v>
       </c>
-      <c r="I23" s="11" t="n">
+      <c r="I23" s="12" t="n">
         <f aca="false">G23*H23</f>
         <v>150</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="14" t="n">
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="15" t="n">
         <f aca="false">SUM(E5:E23)</f>
         <v>8915</v>
       </c>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="14" t="n">
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="15" t="n">
         <f aca="false">SUM(I5:I23)</f>
         <v>18550</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="I25" s="16" t="n">
+      <c r="I25" s="17" t="n">
         <f aca="false">I24-E24</f>
         <v>9635</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="E30" s="18" t="n">
+      <c r="E30" s="19" t="n">
         <f aca="false">E24</f>
         <v>8915</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E31" s="18" t="n">
+      <c r="E31" s="19" t="n">
         <f aca="false">I5-E5</f>
         <v>2586</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="E32" s="20" t="n">
+      <c r="E32" s="21" t="n">
         <f aca="false">E30+E31</f>
         <v>11501</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="B36" s="21" t="s">
+      <c r="B36" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="C36" s="22" t="n">
+      <c r="C36" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D36" s="23" t="n">
+      <c r="D36" s="24" t="n">
         <f aca="false">'Component Options'!$F$13</f>
         <v>1444</v>
       </c>
-      <c r="E36" s="16" t="n">
+      <c r="E36" s="17" t="n">
         <f aca="false">C36*D36</f>
         <v>1444</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="B37" s="21" t="s">
+      <c r="B37" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="C37" s="22" t="n">
+      <c r="C37" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="23" t="n">
+      <c r="D37" s="24" t="n">
         <f aca="false">'Component Options'!$F$17</f>
         <v>3499</v>
       </c>
-      <c r="E37" s="16" t="n">
+      <c r="E37" s="17" t="n">
         <f aca="false">C37*D37-'Component Options'!$F$18</f>
         <v>3000</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="B38" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="C38" s="22" t="n">
+      <c r="C38" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="D38" s="23" t="n">
+      <c r="D38" s="24" t="n">
         <f aca="false">'Component Options'!$F$16</f>
         <v>179</v>
       </c>
-      <c r="E38" s="16" t="n">
+      <c r="E38" s="17" t="n">
         <f aca="false">C38*(D38-'Component Options'!$F$15)</f>
         <v>240</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="19" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="E39" s="24" t="n">
+      <c r="E39" s="25" t="n">
         <f aca="false">SUM(E36:E38)</f>
         <v>4684</v>
       </c>
@@ -3057,552 +3354,1233 @@
   <dimension ref="A1:F38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" s="27" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="B6" s="27" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>180</v>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>885</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" s="27" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B10" s="27" t="n">
+        <v>173</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="B11" s="28" t="n">
+        <f aca="false">'Weight Build-up'!$E$33</f>
+        <v>1144.34734306532</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B12" s="27" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="B14" s="27" t="n">
+        <v>1.225</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="B15" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="B16" s="27" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="B17" s="27" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="B18" s="27" t="n">
+        <v>40</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="B19" s="27" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="B20" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="B21" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="B22" s="27" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="B23" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D23" s="29" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="B24" s="27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D24" s="22" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="B27" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="C27" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="D27" s="26" t="s">
+        <v>227</v>
+      </c>
+      <c r="E27" s="26" t="s">
+        <v>228</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="B28" s="30" t="n">
+        <f aca="false">$B$6*$B$5</f>
+        <v>11100</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>231</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="B29" s="31" t="n">
+        <f aca="false">B28*$B$7*0.0254/60</f>
+        <v>21.1455</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="D29" s="22" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="B30" s="31" t="n">
+        <f aca="false">SQRT(2*$B$11/1000*9.81/($B$14*$B$12*$B$13))</f>
+        <v>7.25722800832826</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="16" t="s">
+        <v>238</v>
+      </c>
+      <c r="B31" s="31" t="n">
+        <f aca="false">B29/B30</f>
+        <v>2.91371581211639</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="D31" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="E31" s="32" t="s">
+        <v>240</v>
+      </c>
+      <c r="F31" s="20" t="str">
+        <f aca="false">IF(B31&gt;=2,"PASS","CHECK")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="B32" s="31" t="n">
+        <f aca="false">$B$8/$B$11</f>
+        <v>0.773366587831089</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D32" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="E32" s="32" t="n">
+        <f aca="false">$B$24</f>
+        <v>0.5</v>
+      </c>
+      <c r="F32" s="20" t="str">
+        <f aca="false">IF(B32&gt;=E32,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="B33" s="31" t="n">
+        <f aca="false">$B$10/($B$11/1000)</f>
+        <v>151.177875361332</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>244</v>
+      </c>
+      <c r="D33" s="22" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="16" t="s">
+        <v>246</v>
+      </c>
+      <c r="B34" s="31" t="n">
+        <f aca="false">$B$15/$B$9</f>
+        <v>1.92307692307692</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="D34" s="22" t="s">
+        <v>247</v>
+      </c>
+      <c r="E34" s="32" t="n">
+        <f aca="false">$B$16</f>
+        <v>1.2</v>
+      </c>
+      <c r="F34" s="20" t="str">
+        <f aca="false">IF(B34&gt;=E34,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="B35" s="31" t="n">
+        <f aca="false">$B$18*$B$17</f>
+        <v>88</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D35" s="22" t="s">
+        <v>249</v>
+      </c>
+      <c r="E35" s="32" t="n">
+        <f aca="false">$B$9</f>
+        <v>15.6</v>
+      </c>
+      <c r="F35" s="20" t="str">
+        <f aca="false">IF(B35&gt;=E35,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="B36" s="31" t="n">
+        <f aca="false">$B$5*$B$17</f>
+        <v>24.42</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="D36" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="E36" s="32" t="s">
+        <v>253</v>
+      </c>
+      <c r="F36" s="20" t="str">
+        <f aca="false">IF(B36&lt;=100,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16" t="s">
+        <v>254</v>
+      </c>
+      <c r="B37" s="31" t="n">
+        <f aca="false">$B$17*$B$19/$B$9*60</f>
+        <v>6.76923076923077</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>255</v>
+      </c>
+      <c r="D37" s="22" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="B38" s="31" t="n">
+        <f aca="false">$B$21*$B$22+$B$23</f>
+        <v>1.1</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>258</v>
+      </c>
+      <c r="E38" s="32" t="n">
+        <f aca="false">$B$20</f>
+        <v>3</v>
+      </c>
+      <c r="F38" s="20" t="str">
+        <f aca="false">IF(B38&lt;=E38,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H43"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>168</v>
+      <c r="A1" s="33" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>169</v>
+      <c r="A2" s="34" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="25" t="s">
-        <v>170</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>173</v>
+      <c r="A4" s="35" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="B5" s="26" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="C5" s="15" t="s">
+      <c r="A5" s="36" t="s">
+        <v>262</v>
+      </c>
+      <c r="B5" s="37" t="n">
+        <v>300</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="36" t="s">
+        <v>264</v>
+      </c>
+      <c r="B6" s="37" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="36" t="s">
+        <v>266</v>
+      </c>
+      <c r="B7" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="36" t="s">
+        <v>268</v>
+      </c>
+      <c r="B8" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="38" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="36" t="s">
+        <v>270</v>
+      </c>
+      <c r="B9" s="37" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="36" t="s">
+        <v>272</v>
+      </c>
+      <c r="B10" s="37" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="36" t="s">
+        <v>274</v>
+      </c>
+      <c r="B11" s="37" t="n">
+        <v>140</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="36" t="s">
+        <v>276</v>
+      </c>
+      <c r="B12" s="37" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="36" t="s">
+        <v>278</v>
+      </c>
+      <c r="B14" s="39" t="n">
+        <f aca="false">PI()/4*($B$7^2-$B$8^2)</f>
+        <v>15.707963267949</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="36" t="s">
+        <v>279</v>
+      </c>
+      <c r="B15" s="39" t="n">
+        <f aca="false">B14*$B$9/1000*$B$10</f>
+        <v>24.3473430653209</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="40" t="s">
+        <v>281</v>
+      </c>
+      <c r="B17" s="40" t="s">
+        <v>282</v>
+      </c>
+      <c r="C17" s="40" t="s">
+        <v>143</v>
+      </c>
+      <c r="D17" s="40" t="s">
+        <v>283</v>
+      </c>
+      <c r="E17" s="40" t="s">
+        <v>284</v>
+      </c>
+      <c r="F17" s="40" t="s">
+        <v>285</v>
+      </c>
+      <c r="G17" s="40" t="s">
+        <v>286</v>
+      </c>
+      <c r="H17" s="40" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="41" t="s">
+        <v>288</v>
+      </c>
+      <c r="B18" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="C18" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="43" t="n">
         <v>175</v>
       </c>
-      <c r="D5" s="21" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="B6" s="26" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="B7" s="26" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D7" s="21" t="s">
+      <c r="E18" s="44" t="n">
+        <f aca="false">C18*D18</f>
+        <v>175</v>
+      </c>
+      <c r="F18" s="45" t="n">
+        <f aca="false">E18/$E$31</f>
+        <v>0.207260674694231</v>
+      </c>
+      <c r="G18" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" s="46" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="41" t="s">
+        <v>291</v>
+      </c>
+      <c r="B19" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="C19" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="E19" s="44" t="n">
+        <f aca="false">C19*D19</f>
+        <v>36</v>
+      </c>
+      <c r="F19" s="45" t="n">
+        <f aca="false">E19/$E$31</f>
+        <v>0.0426364816513847</v>
+      </c>
+      <c r="G19" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19" s="46" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="41" t="s">
+        <v>293</v>
+      </c>
+      <c r="B20" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="C20" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="43" t="n">
+        <v>52</v>
+      </c>
+      <c r="E20" s="44" t="n">
+        <f aca="false">C20*D20</f>
+        <v>52</v>
+      </c>
+      <c r="F20" s="45" t="n">
+        <f aca="false">E20/$E$31</f>
+        <v>0.0615860290520002</v>
+      </c>
+      <c r="G20" s="41" t="s">
+        <v>294</v>
+      </c>
+      <c r="H20" s="46" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="41" t="s">
+        <v>296</v>
+      </c>
+      <c r="B21" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="C21" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="43" t="n">
+        <v>25</v>
+      </c>
+      <c r="E21" s="44" t="n">
+        <f aca="false">C21*D21</f>
+        <v>25</v>
+      </c>
+      <c r="F21" s="45" t="n">
+        <f aca="false">E21/$E$31</f>
+        <v>0.0296086678134616</v>
+      </c>
+      <c r="G21" s="41" t="s">
+        <v>294</v>
+      </c>
+      <c r="H21" s="46" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="41" t="s">
+        <v>298</v>
+      </c>
+      <c r="B22" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="C22" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="E22" s="44" t="n">
+        <f aca="false">C22*D22</f>
+        <v>15</v>
+      </c>
+      <c r="F22" s="45" t="n">
+        <f aca="false">E22/$E$31</f>
+        <v>0.017765200688077</v>
+      </c>
+      <c r="G22" s="41" t="s">
+        <v>294</v>
+      </c>
+      <c r="H22" s="46" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="41" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="B8" s="26" t="n">
-        <v>885</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="B9" s="26" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="B10" s="26" t="n">
-        <v>173</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="B11" s="26" t="n">
-        <v>1144</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>193</v>
-      </c>
-      <c r="B12" s="26" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>194</v>
-      </c>
-      <c r="D12" s="21" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
-        <v>196</v>
-      </c>
-      <c r="B13" s="26" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="D13" s="27" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="B14" s="26" t="n">
-        <v>1.225</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>199</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>201</v>
-      </c>
-      <c r="B15" s="26" t="n">
+      <c r="B23" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="C23" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="43" t="n">
+        <v>12</v>
+      </c>
+      <c r="E23" s="44" t="n">
+        <f aca="false">C23*D23</f>
+        <v>12</v>
+      </c>
+      <c r="F23" s="45" t="n">
+        <f aca="false">E23/$E$31</f>
+        <v>0.0142121605504616</v>
+      </c>
+      <c r="G23" s="41" t="s">
+        <v>294</v>
+      </c>
+      <c r="H23" s="46" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="41" t="s">
+        <v>299</v>
+      </c>
+      <c r="B24" s="41" t="s">
+        <v>300</v>
+      </c>
+      <c r="C24" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="47" t="n">
+        <f aca="false">B15</f>
+        <v>24.3473430653209</v>
+      </c>
+      <c r="E24" s="44" t="n">
+        <f aca="false">C24*D24</f>
+        <v>24.3473430653209</v>
+      </c>
+      <c r="F24" s="45" t="n">
+        <f aca="false">E24/$E$31</f>
+        <v>0.028835695718459</v>
+      </c>
+      <c r="G24" s="41" t="s">
+        <v>301</v>
+      </c>
+      <c r="H24" s="46" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="41" t="s">
+        <v>303</v>
+      </c>
+      <c r="B25" s="41" t="s">
+        <v>300</v>
+      </c>
+      <c r="C25" s="48" t="n">
+        <f aca="false">$B$12</f>
+        <v>2.5</v>
+      </c>
+      <c r="D25" s="47" t="n">
+        <f aca="false">$B$11</f>
+        <v>140</v>
+      </c>
+      <c r="E25" s="44" t="n">
+        <f aca="false">C25*D25</f>
+        <v>350</v>
+      </c>
+      <c r="F25" s="45" t="n">
+        <f aca="false">E25/$E$31</f>
+        <v>0.414521349388463</v>
+      </c>
+      <c r="G25" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="H25" s="46" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="41" t="s">
+        <v>305</v>
+      </c>
+      <c r="B26" s="41" t="s">
+        <v>306</v>
+      </c>
+      <c r="C26" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="E26" s="44" t="n">
+        <f aca="false">C26*D26</f>
+        <v>50</v>
+      </c>
+      <c r="F26" s="45" t="n">
+        <f aca="false">E26/$E$31</f>
+        <v>0.0592173356269232</v>
+      </c>
+      <c r="G26" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="H26" s="46"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="41" t="s">
+        <v>307</v>
+      </c>
+      <c r="B27" s="41" t="s">
+        <v>306</v>
+      </c>
+      <c r="C27" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="43" t="n">
+        <v>40</v>
+      </c>
+      <c r="E27" s="44" t="n">
+        <f aca="false">C27*D27</f>
+        <v>40</v>
+      </c>
+      <c r="F27" s="45" t="n">
+        <f aca="false">E27/$E$31</f>
+        <v>0.0473738685015386</v>
+      </c>
+      <c r="G27" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="H27" s="46"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="41" t="s">
+        <v>308</v>
+      </c>
+      <c r="B28" s="41" t="s">
+        <v>306</v>
+      </c>
+      <c r="C28" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="43" t="n">
         <v>30</v>
       </c>
-      <c r="C15" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
-        <v>203</v>
-      </c>
-      <c r="B16" s="26" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
-        <v>206</v>
-      </c>
-      <c r="B17" s="26" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>207</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
-        <v>209</v>
-      </c>
-      <c r="B18" s="26" t="n">
-        <v>40</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="s">
-        <v>212</v>
-      </c>
-      <c r="B19" s="26" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="D19" s="27" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>214</v>
-      </c>
-      <c r="B20" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
-        <v>216</v>
-      </c>
-      <c r="B21" s="26" t="n">
-        <v>4</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>218</v>
-      </c>
-      <c r="B22" s="26" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C22" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="D22" s="27" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="s">
-        <v>220</v>
-      </c>
-      <c r="B23" s="26" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
-        <v>222</v>
-      </c>
-      <c r="B24" s="26" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25" t="s">
-        <v>225</v>
-      </c>
-      <c r="B27" s="25" t="s">
-        <v>226</v>
-      </c>
-      <c r="C27" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="D27" s="25" t="s">
-        <v>227</v>
-      </c>
-      <c r="E27" s="25" t="s">
-        <v>228</v>
-      </c>
-      <c r="F27" s="25" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
-        <v>230</v>
-      </c>
-      <c r="B28" s="28" t="n">
-        <f aca="false">$B$6*$B$5</f>
-        <v>11100</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>231</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>232</v>
-      </c>
+      <c r="E28" s="44" t="n">
+        <f aca="false">C28*D28</f>
+        <v>30</v>
+      </c>
+      <c r="F28" s="45" t="n">
+        <f aca="false">E28/$E$31</f>
+        <v>0.0355304013761539</v>
+      </c>
+      <c r="G28" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="H28" s="46"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
-        <v>233</v>
-      </c>
-      <c r="B29" s="29" t="n">
-        <f aca="false">B28*$B$7*0.0254/60</f>
-        <v>21.1455</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>234</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>235</v>
-      </c>
+      <c r="A29" s="41" t="s">
+        <v>309</v>
+      </c>
+      <c r="B29" s="41" t="s">
+        <v>306</v>
+      </c>
+      <c r="C29" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="E29" s="44" t="n">
+        <f aca="false">C29*D29</f>
+        <v>15</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <f aca="false">E29/$E$31</f>
+        <v>0.017765200688077</v>
+      </c>
+      <c r="G29" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="H29" s="46"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
-        <v>236</v>
-      </c>
-      <c r="B30" s="29" t="n">
-        <f aca="false">SQRT(2*$B$11/1000*9.81/($B$14*$B$12*$B$13))</f>
-        <v>7.25612653369876</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>234</v>
-      </c>
-      <c r="D30" s="21" t="s">
-        <v>237</v>
-      </c>
+      <c r="A30" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="B30" s="41" t="s">
+        <v>306</v>
+      </c>
+      <c r="C30" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="43" t="n">
+        <v>20</v>
+      </c>
+      <c r="E30" s="44" t="n">
+        <f aca="false">C30*D30</f>
+        <v>20</v>
+      </c>
+      <c r="F30" s="45" t="n">
+        <f aca="false">E30/$E$31</f>
+        <v>0.0236869342507693</v>
+      </c>
+      <c r="G30" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="H30" s="46"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
-        <v>238</v>
-      </c>
-      <c r="B31" s="29" t="n">
-        <f aca="false">B29/B30</f>
-        <v>2.914158112017</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>239</v>
-      </c>
-      <c r="E31" s="30" t="s">
-        <v>240</v>
-      </c>
-      <c r="F31" s="19" t="str">
-        <f aca="false">IF(B31&gt;=2,"PASS","CHECK")</f>
-        <v>PASS</v>
-      </c>
+      <c r="A31" s="49" t="s">
+        <v>310</v>
+      </c>
+      <c r="B31" s="50"/>
+      <c r="C31" s="50"/>
+      <c r="D31" s="50"/>
+      <c r="E31" s="51" t="n">
+        <f aca="false">SUM(E18:E30)</f>
+        <v>844.347343065321</v>
+      </c>
+      <c r="F31" s="50"/>
+      <c r="G31" s="50"/>
+      <c r="H31" s="50"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="s">
-        <v>241</v>
-      </c>
-      <c r="B32" s="29" t="n">
-        <f aca="false">$B$8/$B$11</f>
-        <v>0.773601398601399</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>242</v>
-      </c>
-      <c r="E32" s="30" t="n">
-        <f aca="false">$B$24</f>
-        <v>0.5</v>
-      </c>
-      <c r="F32" s="19" t="str">
-        <f aca="false">IF(B32&gt;=E32,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
+      <c r="A32" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="B32" s="50"/>
+      <c r="C32" s="50"/>
+      <c r="D32" s="50"/>
+      <c r="E32" s="52" t="n">
+        <f aca="false">$B$5</f>
+        <v>300</v>
+      </c>
+      <c r="F32" s="50"/>
+      <c r="G32" s="50"/>
+      <c r="H32" s="50"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="s">
-        <v>243</v>
-      </c>
-      <c r="B33" s="29" t="n">
-        <f aca="false">$B$10/($B$11/1000)</f>
-        <v>151.223776223776</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="D33" s="21" t="s">
-        <v>245</v>
-      </c>
+      <c r="A33" s="49" t="s">
+        <v>312</v>
+      </c>
+      <c r="B33" s="50"/>
+      <c r="C33" s="50"/>
+      <c r="D33" s="50"/>
+      <c r="E33" s="53" t="n">
+        <f aca="false">E31+E32</f>
+        <v>1144.34734306532</v>
+      </c>
+      <c r="F33" s="50"/>
+      <c r="G33" s="50"/>
+      <c r="H33" s="50"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15" t="s">
-        <v>246</v>
-      </c>
-      <c r="B34" s="29" t="n">
-        <f aca="false">$B$15/$B$9</f>
-        <v>1.92307692307692</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="D34" s="21" t="s">
-        <v>247</v>
-      </c>
-      <c r="E34" s="30" t="n">
-        <f aca="false">$B$16</f>
-        <v>1.2</v>
-      </c>
-      <c r="F34" s="19" t="str">
-        <f aca="false">IF(B34&gt;=E34,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
+      <c r="A34" s="49" t="s">
+        <v>313</v>
+      </c>
+      <c r="B34" s="50"/>
+      <c r="C34" s="50"/>
+      <c r="D34" s="50"/>
+      <c r="E34" s="52" t="n">
+        <f aca="false">$B$6</f>
+        <v>1200</v>
+      </c>
+      <c r="F34" s="50"/>
+      <c r="G34" s="50"/>
+      <c r="H34" s="50"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="s">
-        <v>248</v>
-      </c>
-      <c r="B35" s="29" t="n">
-        <f aca="false">$B$18*$B$17</f>
-        <v>88</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="D35" s="21" t="s">
-        <v>249</v>
-      </c>
-      <c r="E35" s="30" t="n">
-        <f aca="false">$B$9</f>
-        <v>15.6</v>
-      </c>
-      <c r="F35" s="19" t="str">
-        <f aca="false">IF(B35&gt;=E35,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
+      <c r="A35" s="49" t="s">
+        <v>314</v>
+      </c>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
+      <c r="E35" s="51" t="n">
+        <f aca="false">E34-E33</f>
+        <v>55.6526569346793</v>
+      </c>
+      <c r="F35" s="50"/>
+      <c r="G35" s="50"/>
+      <c r="H35" s="50"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15" t="s">
-        <v>250</v>
-      </c>
-      <c r="B36" s="29" t="n">
-        <f aca="false">$B$5*$B$17</f>
-        <v>24.42</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>251</v>
-      </c>
-      <c r="D36" s="21" t="s">
-        <v>252</v>
-      </c>
-      <c r="E36" s="30" t="s">
-        <v>253</v>
-      </c>
-      <c r="F36" s="19" t="str">
-        <f aca="false">IF(B36&lt;=100,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="s">
-        <v>254</v>
-      </c>
-      <c r="B37" s="29" t="n">
-        <f aca="false">$B$17*$B$19/$B$9*60</f>
-        <v>6.76923076923077</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>255</v>
-      </c>
-      <c r="D37" s="21" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="s">
-        <v>257</v>
-      </c>
-      <c r="B38" s="29" t="n">
-        <f aca="false">$B$21*$B$22+$B$23</f>
-        <v>1.1</v>
-      </c>
-      <c r="C38" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="D38" s="21" t="s">
-        <v>258</v>
-      </c>
-      <c r="E38" s="30" t="n">
-        <f aca="false">$B$20</f>
-        <v>3</v>
-      </c>
-      <c r="F38" s="19" t="str">
-        <f aca="false">IF(B38&lt;=E38,"PASS","FAIL")</f>
-        <v>PASS</v>
+      <c r="A36" s="49" t="s">
+        <v>315</v>
+      </c>
+      <c r="B36" s="50"/>
+      <c r="C36" s="50"/>
+      <c r="D36" s="50"/>
+      <c r="E36" s="54" t="n">
+        <f aca="false">IF(E34=0,0,E35/E34)</f>
+        <v>0.0463772141122327</v>
+      </c>
+      <c r="F36" s="50"/>
+      <c r="G36" s="50"/>
+      <c r="H36" s="50"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="35" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="55" t="s">
+        <v>282</v>
+      </c>
+      <c r="B40" s="55" t="s">
+        <v>317</v>
+      </c>
+      <c r="C40" s="55" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="B41" s="44" t="n">
+        <f aca="false">SUMIF($B$18:$B$30,A41,$E$18:$E$30)</f>
+        <v>315</v>
+      </c>
+      <c r="C41" s="45" t="n">
+        <f aca="false">B41/$E$31</f>
+        <v>0.373069214449616</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="41" t="s">
+        <v>300</v>
+      </c>
+      <c r="B42" s="44" t="n">
+        <f aca="false">SUMIF($B$18:$B$30,A42,$E$18:$E$30)</f>
+        <v>374.347343065321</v>
+      </c>
+      <c r="C42" s="45" t="n">
+        <f aca="false">B42/$E$31</f>
+        <v>0.443357045106922</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="41" t="s">
+        <v>306</v>
+      </c>
+      <c r="B43" s="44" t="n">
+        <f aca="false">SUMIF($B$18:$B$30,A43,$E$18:$E$30)</f>
+        <v>155</v>
+      </c>
+      <c r="C43" s="45" t="n">
+        <f aca="false">B43/$E$31</f>
+        <v>0.183573740443462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>